<commit_message>
Add target-headcount solver and second-DJ tier to the door-split calculator
- docs/dj-pay.html: new "Hit the cap at a target headcount" section
  back-solves the split %, guarantee, or cap needed for the DJ to hit
  the cap at a chosen headcount and cover charge, with an Apply button
  that writes the result into Deal terms.
- docs/dj-pay.html: new "Second DJ" section models DJ1's guarantee ->
  DJ2's flat cut -> back to the DJ1/house split until DJ1 caps -> house
  keeps the rest, with its own tier breakdown and headcount grid.
- docs/dj-pay.xlsx: mirrors both features with live formulas — a
  target-headcount solver block on the DJ Pay sheet (three options:
  adjust split/guarantee/cap) and a new "Two DJs" sheet with the same
  tiered model, a self-checking tier table, and a headcount grid.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ed5kV3pbHKvNoecFDSmMGp
</commit_message>
<xml_diff>
--- a/docs/dj-pay.xlsx
+++ b/docs/dj-pay.xlsx
@@ -9,6 +9,7 @@
   </bookViews>
   <sheets>
     <sheet name="DJ Pay" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Two DJs" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="72">
   <si>
     <t xml:space="preserve">Azúcar · DJ Door Split</t>
   </si>
@@ -140,6 +141,102 @@
   </si>
   <si>
     <t xml:space="preserve">Rule: first $200 at the door goes to the DJ, then 50/50 until the DJ reaches $500, then 100% to you. Amounts come from your deal with the DJ.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HIT THE CAP AT A TARGET HEADCOUNT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pick a headcount you want the DJ to reach the cap at. Each row below solves for the one deal term that gets you there, holding the other two fixed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target headcount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">At this cover charge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Door total at target</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adjust</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lower the split (keep guarantee &amp; cap)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Change the guarantee (keep split &amp; cap)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Change the cap (keep guarantee &amp; split)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pick one option and type it into Deal Terms above (B9, B10 or B11) — the sheet recalculates everything else.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Azúcar · Two DJs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DJ1 gets his first dollars → DJ2 gets his cut → back to the DJ1/house split until DJ1 caps → then it's all yours.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DJ1's first dollars (100% to DJ1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DJ2's pay is a flat cut — it isn't capped separately, it's just this one amount.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DJ2's cut, right after that (100% to DJ2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DJ1 share after DJ2 is paid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DJ1 cap for the night</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DJ1 gets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DJ2 gets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Door total at which DJ1 is capped</t>
+  </si>
+  <si>
+    <t xml:space="preserve">People needed to cap DJ1 at this cover</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DJ1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DJ2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DJ1 / DJ2 / YOU BY HEADCOUNT (AT TONIGHT'S COVER)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">People</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Door</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Headcounts in column A are editable. Each row uses tonight's cover charge (B5).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DJ1's money</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DJ2's money</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rule: DJ1's first dollars go 100% to DJ1, then DJ2's cut goes 100% to DJ2, then it's back to DJ1's split with the house until DJ1 hits his cap — after that, everything is yours.</t>
   </si>
 </sst>
 </file>
@@ -221,7 +318,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -249,7 +346,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFEEEEEE"/>
-        <bgColor rgb="FFFFF1D6"/>
+        <bgColor rgb="FFDCEEFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCEEFF"/>
+        <bgColor rgb="FFEEEEEE"/>
       </patternFill>
     </fill>
   </fills>
@@ -302,7 +405,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -404,6 +507,22 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -437,7 +556,7 @@
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFF1D6"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFDCEEFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
@@ -659,7 +778,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -1485,6 +1604,660 @@
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B64" s="6" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B65" s="5" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B66" s="8" t="n">
+        <f aca="false">$B$64*$B$65</f>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="B68" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="C68" s="14"/>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B69" s="26" t="str">
+        <f aca="false">IF($B$66&lt;=$B$9,"n/a - inside guarantee",IF($B$11&lt;=$B$9,"n/a - cap below guarantee",IF((($B$11-$B$9)/($B$66-$B$9))&gt;1,"not possible (&gt;100%)",IF((($B$11-$B$9)/($B$66-$B$9))&lt;=0,"not possible (&lt;=0%)",TEXT(ROUND((($B$11-$B$9)/($B$66-$B$9))*100,1),"0.0")&amp;"%"))))</f>
+        <v>37.5%</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B70" s="26" t="str">
+        <f aca="false">IF($B$10&gt;=1,"n/a - split is 100%",IF((($B$11-$B$10*$B$66)/(1-$B$10))&lt;0,"not possible (&lt;$0)",IF((($B$11-$B$10*$B$66)/(1-$B$10))&gt;$B$11,"not possible (&gt;cap)","$"&amp;TEXT(ROUND(($B$11-$B$10*$B$66)/(1-$B$10),0),"#,##0"))))</f>
+        <v>$0</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B71" s="26" t="str">
+        <f aca="false">IF(($B$9+$B$10*($B$66-$B$9))&lt;$B$9,"not possible","$"&amp;TEXT(ROUND($B$9+$B$10*($B$66-$B$9),0),"#,##0"))</f>
+        <v>$600</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E51"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>200</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="8" t="n">
+        <f aca="false">B5*B6</f>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" s="9" t="n">
+        <f aca="false">MIN(MIN($B$9,B15)+IF($B$11&gt;0,MIN(MAX(0,MAX(0,B15-$B$9)-$B$10)*$B$11,MAX(0,$B$12-MIN($B$9,B15))),0),$B$12)</f>
+        <v>500</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B17" s="27" t="n">
+        <f aca="false">MIN(MAX(0,B15-$B$9),$B$10)</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" s="10" t="n">
+        <f aca="false">B15-B16-B17</f>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B19" s="11" t="n">
+        <f aca="false">IF(B12&lt;=B9,B12,IF(B11&lt;=0,"never",B9+B10+(B12-B9)/B11))</f>
+        <v>900</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B20" s="12" t="n">
+        <f aca="false">IF(OR(B5&lt;=0,NOT(ISNUMBER(B19))),"never",ROUNDUP(B19/B5,0))</f>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21" s="4" t="str">
+        <f aca="false">IF(B15=0,"No door yet",IF(B16&gt;=B12,"DJ1 capped, DJ2 paid in full, rest is yours",IF(B15&lt;=B9,"Still inside DJ1's first $"&amp;TEXT(B9,"0"),IF(B15&lt;=B9+B10,"DJ1 covered, now inside DJ2's cut","DJ1 is $"&amp;TEXT(B12-B16,"0")&amp;" short of cap"))))</f>
+        <v>DJ1 capped, DJ2 paid in full, rest is yours</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="D24" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="str">
+        <f aca="false">"First $"&amp;TEXT(B9,"0")&amp;" (100% to DJ1)"</f>
+        <v>First $200 (100% to DJ1)</v>
+      </c>
+      <c r="B25" s="11" t="n">
+        <f aca="false">MIN(B15,B9)</f>
+        <v>200</v>
+      </c>
+      <c r="C25" s="15" t="n">
+        <f aca="false">B25</f>
+        <v>200</v>
+      </c>
+      <c r="D25" s="28" t="n">
+        <f aca="false">0</f>
+        <v>0</v>
+      </c>
+      <c r="E25" s="16" t="n">
+        <f aca="false">0</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="str">
+        <f aca="false">"Next $"&amp;TEXT(B10,"0")&amp;" (100% to DJ2)"</f>
+        <v>Next $100 (100% to DJ2)</v>
+      </c>
+      <c r="B26" s="11" t="n">
+        <f aca="false">MAX(0,MIN(B15-B9,B10))</f>
+        <v>100</v>
+      </c>
+      <c r="C26" s="15" t="n">
+        <f aca="false">0</f>
+        <v>0</v>
+      </c>
+      <c r="D26" s="28" t="n">
+        <f aca="false">B26</f>
+        <v>100</v>
+      </c>
+      <c r="E26" s="16" t="n">
+        <f aca="false">0</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="str">
+        <f aca="false">"Then (DJ1 "&amp;TEXT(B11,"0%")&amp;" / you "&amp;TEXT(1-B11,"0%")&amp;")"</f>
+        <v>Then (DJ1 50% / you 50%)</v>
+      </c>
+      <c r="B27" s="11" t="n">
+        <f aca="false">IF(ISNUMBER(B19),MAX(0,MIN(B15-B9-B10,B19-B9-B10)),MAX(0,B15-B9-B10))</f>
+        <v>600</v>
+      </c>
+      <c r="C27" s="15" t="n">
+        <f aca="false">B27*B11</f>
+        <v>300</v>
+      </c>
+      <c r="D27" s="28" t="n">
+        <f aca="false">0</f>
+        <v>0</v>
+      </c>
+      <c r="E27" s="16" t="n">
+        <f aca="false">B27-C27</f>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="str">
+        <f aca="false">IF(ISNUMBER(B19),"Above $"&amp;TEXT(B19,"0")&amp;" (DJ1 capped, 100% to you)","Above cap (n/a)")</f>
+        <v>Above $900 (DJ1 capped, 100% to you)</v>
+      </c>
+      <c r="B28" s="11" t="n">
+        <f aca="false">IF(ISNUMBER(B19),MAX(0,B15-B19),0)</f>
+        <v>100</v>
+      </c>
+      <c r="C28" s="15" t="n">
+        <f aca="false">0</f>
+        <v>0</v>
+      </c>
+      <c r="D28" s="28" t="n">
+        <f aca="false">0</f>
+        <v>0</v>
+      </c>
+      <c r="E28" s="16" t="n">
+        <f aca="false">B28</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B29" s="8" t="n">
+        <f aca="false">SUM(B25:B28)</f>
+        <v>1000</v>
+      </c>
+      <c r="C29" s="9" t="n">
+        <f aca="false">SUM(C25:C28)</f>
+        <v>500</v>
+      </c>
+      <c r="D29" s="27" t="n">
+        <f aca="false">SUM(D25:D28)</f>
+        <v>100</v>
+      </c>
+      <c r="E29" s="10" t="n">
+        <f aca="false">SUM(E25:E28)</f>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="str">
+        <f aca="false">IF(AND(ROUND(C29-B16,2)=0,ROUND(D29-B17,2)=0),"check ok","CHECK: tiers do not match the split above")</f>
+        <v>check ok</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="B33" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C33" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="D33" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="E33" s="14" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="B34" s="20" t="n">
+        <f aca="false">A34*$B$5</f>
+        <v>50</v>
+      </c>
+      <c r="C34" s="20" t="n">
+        <f aca="false">MIN(MIN($B$9,B34)+IF($B$11&gt;0,MIN(MAX(0,MAX(0,B34-$B$9)-$B$10)*$B$11,MAX(0,$B$12-MIN($B$9,B34))),0),$B$12)</f>
+        <v>50</v>
+      </c>
+      <c r="D34" s="20" t="n">
+        <f aca="false">MIN(MAX(0,B34-$B$9),$B$10)</f>
+        <v>0</v>
+      </c>
+      <c r="E34" s="20" t="n">
+        <f aca="false">B34-C34-D34</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="B35" s="20" t="n">
+        <f aca="false">A35*$B$5</f>
+        <v>100</v>
+      </c>
+      <c r="C35" s="20" t="n">
+        <f aca="false">MIN(MIN($B$9,B35)+IF($B$11&gt;0,MIN(MAX(0,MAX(0,B35-$B$9)-$B$10)*$B$11,MAX(0,$B$12-MIN($B$9,B35))),0),$B$12)</f>
+        <v>100</v>
+      </c>
+      <c r="D35" s="20" t="n">
+        <f aca="false">MIN(MAX(0,B35-$B$9),$B$10)</f>
+        <v>0</v>
+      </c>
+      <c r="E35" s="20" t="n">
+        <f aca="false">B35-C35-D35</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="22" t="n">
+        <v>20</v>
+      </c>
+      <c r="B36" s="20" t="n">
+        <f aca="false">A36*$B$5</f>
+        <v>200</v>
+      </c>
+      <c r="C36" s="20" t="n">
+        <f aca="false">MIN(MIN($B$9,B36)+IF($B$11&gt;0,MIN(MAX(0,MAX(0,B36-$B$9)-$B$10)*$B$11,MAX(0,$B$12-MIN($B$9,B36))),0),$B$12)</f>
+        <v>200</v>
+      </c>
+      <c r="D36" s="20" t="n">
+        <f aca="false">MIN(MAX(0,B36-$B$9),$B$10)</f>
+        <v>0</v>
+      </c>
+      <c r="E36" s="20" t="n">
+        <f aca="false">B36-C36-D36</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="22" t="n">
+        <v>30</v>
+      </c>
+      <c r="B37" s="20" t="n">
+        <f aca="false">A37*$B$5</f>
+        <v>300</v>
+      </c>
+      <c r="C37" s="20" t="n">
+        <f aca="false">MIN(MIN($B$9,B37)+IF($B$11&gt;0,MIN(MAX(0,MAX(0,B37-$B$9)-$B$10)*$B$11,MAX(0,$B$12-MIN($B$9,B37))),0),$B$12)</f>
+        <v>200</v>
+      </c>
+      <c r="D37" s="20" t="n">
+        <f aca="false">MIN(MAX(0,B37-$B$9),$B$10)</f>
+        <v>100</v>
+      </c>
+      <c r="E37" s="20" t="n">
+        <f aca="false">B37-C37-D37</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="22" t="n">
+        <v>40</v>
+      </c>
+      <c r="B38" s="20" t="n">
+        <f aca="false">A38*$B$5</f>
+        <v>400</v>
+      </c>
+      <c r="C38" s="20" t="n">
+        <f aca="false">MIN(MIN($B$9,B38)+IF($B$11&gt;0,MIN(MAX(0,MAX(0,B38-$B$9)-$B$10)*$B$11,MAX(0,$B$12-MIN($B$9,B38))),0),$B$12)</f>
+        <v>250</v>
+      </c>
+      <c r="D38" s="20" t="n">
+        <f aca="false">MIN(MAX(0,B38-$B$9),$B$10)</f>
+        <v>100</v>
+      </c>
+      <c r="E38" s="20" t="n">
+        <f aca="false">B38-C38-D38</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="22" t="n">
+        <v>50</v>
+      </c>
+      <c r="B39" s="20" t="n">
+        <f aca="false">A39*$B$5</f>
+        <v>500</v>
+      </c>
+      <c r="C39" s="20" t="n">
+        <f aca="false">MIN(MIN($B$9,B39)+IF($B$11&gt;0,MIN(MAX(0,MAX(0,B39-$B$9)-$B$10)*$B$11,MAX(0,$B$12-MIN($B$9,B39))),0),$B$12)</f>
+        <v>300</v>
+      </c>
+      <c r="D39" s="20" t="n">
+        <f aca="false">MIN(MAX(0,B39-$B$9),$B$10)</f>
+        <v>100</v>
+      </c>
+      <c r="E39" s="20" t="n">
+        <f aca="false">B39-C39-D39</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="22" t="n">
+        <v>75</v>
+      </c>
+      <c r="B40" s="20" t="n">
+        <f aca="false">A40*$B$5</f>
+        <v>750</v>
+      </c>
+      <c r="C40" s="20" t="n">
+        <f aca="false">MIN(MIN($B$9,B40)+IF($B$11&gt;0,MIN(MAX(0,MAX(0,B40-$B$9)-$B$10)*$B$11,MAX(0,$B$12-MIN($B$9,B40))),0),$B$12)</f>
+        <v>425</v>
+      </c>
+      <c r="D40" s="20" t="n">
+        <f aca="false">MIN(MAX(0,B40-$B$9),$B$10)</f>
+        <v>100</v>
+      </c>
+      <c r="E40" s="20" t="n">
+        <f aca="false">B40-C40-D40</f>
+        <v>225</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="22" t="n">
+        <v>100</v>
+      </c>
+      <c r="B41" s="20" t="n">
+        <f aca="false">A41*$B$5</f>
+        <v>1000</v>
+      </c>
+      <c r="C41" s="20" t="n">
+        <f aca="false">MIN(MIN($B$9,B41)+IF($B$11&gt;0,MIN(MAX(0,MAX(0,B41-$B$9)-$B$10)*$B$11,MAX(0,$B$12-MIN($B$9,B41))),0),$B$12)</f>
+        <v>500</v>
+      </c>
+      <c r="D41" s="20" t="n">
+        <f aca="false">MIN(MAX(0,B41-$B$9),$B$10)</f>
+        <v>100</v>
+      </c>
+      <c r="E41" s="20" t="n">
+        <f aca="false">B41-C41-D41</f>
+        <v>400</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="22" t="n">
+        <v>150</v>
+      </c>
+      <c r="B42" s="20" t="n">
+        <f aca="false">A42*$B$5</f>
+        <v>1500</v>
+      </c>
+      <c r="C42" s="20" t="n">
+        <f aca="false">MIN(MIN($B$9,B42)+IF($B$11&gt;0,MIN(MAX(0,MAX(0,B42-$B$9)-$B$10)*$B$11,MAX(0,$B$12-MIN($B$9,B42))),0),$B$12)</f>
+        <v>500</v>
+      </c>
+      <c r="D42" s="20" t="n">
+        <f aca="false">MIN(MAX(0,B42-$B$9),$B$10)</f>
+        <v>100</v>
+      </c>
+      <c r="E42" s="20" t="n">
+        <f aca="false">B42-C42-D42</f>
+        <v>900</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="22" t="n">
+        <v>200</v>
+      </c>
+      <c r="B43" s="20" t="n">
+        <f aca="false">A43*$B$5</f>
+        <v>2000</v>
+      </c>
+      <c r="C43" s="20" t="n">
+        <f aca="false">MIN(MIN($B$9,B43)+IF($B$11&gt;0,MIN(MAX(0,MAX(0,B43-$B$9)-$B$10)*$B$11,MAX(0,$B$12-MIN($B$9,B43))),0),$B$12)</f>
+        <v>500</v>
+      </c>
+      <c r="D43" s="20" t="n">
+        <f aca="false">MIN(MAX(0,B43-$B$9),$B$10)</f>
+        <v>100</v>
+      </c>
+      <c r="E43" s="20" t="n">
+        <f aca="false">B43-C43-D43</f>
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="29" t="s">
+        <v>69</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="2" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>